<commit_message>
Fix Q4 reference CSV formatting and workbook opening sheet
</commit_message>
<xml_diff>
--- a/docs/SIH_SUS_2024_Variable_Selection_and_Analysis_Plan.xlsx
+++ b/docs/SIH_SUS_2024_Variable_Selection_and_Analysis_Plan.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Practice_projects\01_sis-suh\github\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Practice_projects\01_sis-suh\SIH_SUS_2024_github\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072"/>
   </bookViews>
   <sheets>
     <sheet name="final_list" sheetId="7" r:id="rId1"/>

</xml_diff>